<commit_message>
Generalise anonymisation placeholder, restore redact-at-source instruction
</commit_message>
<xml_diff>
--- a/submissions/log-cowork-session-cost/assets/cowork-cost-log-template.xlsx
+++ b/submissions/log-cowork-session-cost/assets/cowork-cost-log-template.xlsx
@@ -1102,7 +1102,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Project / Context: What the session was for, with the client name anonymised, for example "[Client] CRM".</t>
+          <t>Project / Context: What the session was for, with the client name anonymised, in the form "[Client] [Task]".</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>Never name the actual client or organisation anywhere in this workbook, including the Project / Context and the commentary columns. Use a generic placeholder that still conveys the type of work, for example "[Client] CRM" or "a higher education client's case management project".</t>
+          <t>Never name the actual client or organisation anywhere in this workbook, including the Project / Context and the commentary columns. Use a generic placeholder that still conveys the type of work, in the form "[Client] [Task]".</t>
         </is>
       </c>
     </row>
@@ -1483,13 +1483,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8195F7D-5706-4338-B1E8-0E6BBDA14393}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8141F461-0369-414B-B319-3FE93A313AF8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC8DF3FC-AB65-43DE-8793-5B72DFBE92C9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1271F924-4576-4067-A4EE-3D427B2AAE64}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{189B1E9D-6D41-4047-9566-9BA82D868033}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9D86445-8D29-403E-A670-F190E5763FB5}"/>
 </file>
</xml_diff>